<commit_message>
Update Reference_NMB_copy1.xlsx and modify columns to keep in data processing
</commit_message>
<xml_diff>
--- a/apollodata/Reference_NMB_copy1.xlsx
+++ b/apollodata/Reference_NMB_copy1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AskPoorni\Svyasa\NMB_data\Apollo data\team ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D41074-0AE1-430B-81F0-EF33C517CF48}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74986FCE-7E2B-4695-BF75-6424FD224EFE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17544" windowHeight="7968" xr2:uid="{5CAC90CE-3BD8-4DB6-BA32-A6D0BF4ECD9E}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="194">
   <si>
     <t>PostRgroupname</t>
   </si>
@@ -563,36 +563,6 @@
   </si>
   <si>
     <t>or else impute diabetic duration as 0</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Create a new column as </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>systolic</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Create a new column as </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>diastolic</t>
-    </r>
   </si>
   <si>
     <t>PreRsystolicfirst or PreRsystolicsecond(whichever is higher)</t>
@@ -1575,7 +1545,7 @@
         <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>87</v>
@@ -1583,7 +1553,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>113</v>
@@ -1591,10 +1561,10 @@
     </row>
     <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D4" t="s">
         <v>88</v>
@@ -1602,34 +1572,34 @@
     </row>
     <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>89</v>
@@ -1637,10 +1607,10 @@
     </row>
     <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>90</v>
@@ -1656,10 +1626,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1667,7 +1637,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1675,7 +1645,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1683,7 +1653,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1706,13 +1676,13 @@
         <v>9</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C23" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D23" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1742,7 +1712,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1762,7 +1732,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -1775,7 +1745,7 @@
         <v>19</v>
       </c>
       <c r="C36" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
@@ -1783,10 +1753,10 @@
         <v>20</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D37" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
@@ -1822,14 +1792,14 @@
     </row>
     <row r="45" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D45" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -1954,10 +1924,10 @@
     </row>
     <row r="64" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C64" s="7"/>
       <c r="D64" s="7"/>
@@ -1969,13 +1939,13 @@
         <v>53</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C65" s="8"/>
       <c r="D65" s="8"/>
       <c r="E65" s="9"/>
       <c r="G65" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H65" s="16" t="s">
         <v>97</v>
@@ -1992,10 +1962,10 @@
     </row>
     <row r="66" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C66" s="8"/>
       <c r="D66" s="8"/>
@@ -2011,7 +1981,7 @@
         <v>54</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C67" s="8"/>
       <c r="D67" s="8"/>
@@ -2027,10 +1997,10 @@
     </row>
     <row r="68" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C68" s="8"/>
       <c r="D68" s="8"/>
@@ -2042,7 +2012,7 @@
         <v>55</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C69" s="8"/>
       <c r="D69" s="8"/>
@@ -2126,7 +2096,7 @@
         <v>59</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F76" t="s">
         <v>70</v>
@@ -2137,7 +2107,7 @@
         <v>60</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F77" t="s">
         <v>70</v>
@@ -2148,7 +2118,7 @@
         <v>61</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F78" t="s">
         <v>70</v>
@@ -2159,7 +2129,7 @@
         <v>62</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F79" t="s">
         <v>70</v>
@@ -2170,7 +2140,7 @@
         <v>63</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F80" t="s">
         <v>71</v>
@@ -2181,7 +2151,7 @@
         <v>64</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F81" t="s">
         <v>70</v>
@@ -2192,7 +2162,7 @@
         <v>65</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F82" t="s">
         <v>70</v>
@@ -2203,7 +2173,7 @@
         <v>66</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F83" t="s">
         <v>70</v>
@@ -2214,7 +2184,7 @@
         <v>67</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F84" t="s">
         <v>70</v>
@@ -2225,7 +2195,7 @@
         <v>68</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F85" t="s">
         <v>70</v>
@@ -2236,13 +2206,13 @@
         <v>69</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C86" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
@@ -2260,7 +2230,7 @@
         <v>73</v>
       </c>
       <c r="B91" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
@@ -2295,7 +2265,7 @@
         <v>113</v>
       </c>
       <c r="D95" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>81</v>
@@ -2320,55 +2290,49 @@
       </c>
     </row>
     <row r="101" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A101" s="2" t="s">
+      <c r="A101" t="s">
+        <v>180</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G101" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="B101" t="s">
-        <v>182</v>
-      </c>
-      <c r="D101" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F101" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G101" s="2" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D102" s="2"/>
       <c r="F102" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A103" s="2" t="s">
+      <c r="A103" t="s">
+        <v>181</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G103" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="B103" t="s">
-        <v>183</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F103" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G103" s="2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D104" s="10"/>
       <c r="F104" t="s">
+        <v>136</v>
+      </c>
+      <c r="G104" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="G104" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.3">
@@ -2456,10 +2420,10 @@
         <v>118</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E121" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F121" s="2" t="s">
         <v>125</v>
@@ -2490,18 +2454,18 @@
         <v>128</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E125" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F125" s="23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F128" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>